<commit_message>
SPM-36: Record manual test run (7 pass)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-36_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-36_Test_Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janelleip/Documents/GitHub/IS212/docs/test-cases/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krist\Documents\GitHub\IS212\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C539D3F1-71F2-764F-982A-D01EB3F4D845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2384180D-92A1-409C-9EF5-04E2A46110EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="110">
   <si>
     <t>Story</t>
   </si>
@@ -404,6 +404,9 @@
   <si>
     <t>ebf85f1</t>
   </si>
+  <si>
+    <t>Kristen</t>
+  </si>
 </sst>
 </file>
 
@@ -412,7 +415,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -452,6 +455,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -478,7 +488,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -540,11 +550,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -570,14 +593,21 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -794,7 +824,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -807,11 +837,11 @@
     <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:9" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="14"/>
@@ -822,7 +852,7 @@
       <c r="H1" s="14"/>
       <c r="I1" s="15"/>
     </row>
-    <row r="3" spans="1:9" ht="14" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
@@ -851,7 +881,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="42" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:9" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>11</v>
       </c>
@@ -876,7 +906,7 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
     </row>
-    <row r="5" spans="1:9" ht="28" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
@@ -901,7 +931,7 @@
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
     </row>
-    <row r="6" spans="1:9" ht="28" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>22</v>
       </c>
@@ -926,7 +956,7 @@
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
     </row>
-    <row r="7" spans="1:9" ht="28" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>27</v>
       </c>
@@ -951,7 +981,7 @@
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
     </row>
-    <row r="8" spans="1:9" ht="42" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:9" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>31</v>
       </c>
@@ -976,7 +1006,7 @@
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
     </row>
-    <row r="9" spans="1:9" ht="42" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:9" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>35</v>
       </c>
@@ -1001,7 +1031,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="10" spans="1:9" ht="28" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>39</v>
       </c>
@@ -1026,109 +1056,109 @@
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
     </row>
-    <row r="13" spans="1:9" ht="14" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="13" t="s">
         <v>45</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="15"/>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="13" t="s">
         <v>46</v>
       </c>
       <c r="F13" s="15"/>
     </row>
-    <row r="14" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:9" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="16" t="s">
         <v>47</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="15"/>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="16" t="s">
         <v>48</v>
       </c>
       <c r="F14" s="15"/>
     </row>
-    <row r="15" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="16" t="s">
         <v>50</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="15"/>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="16" t="s">
         <v>51</v>
       </c>
       <c r="F15" s="15"/>
     </row>
-    <row r="16" spans="1:9" ht="58" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:9" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="16" t="s">
         <v>53</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="15"/>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="16" t="s">
         <v>54</v>
       </c>
       <c r="F16" s="15"/>
     </row>
-    <row r="17" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="16" t="s">
         <v>56</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="15"/>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F17" s="15"/>
     </row>
-    <row r="18" spans="1:9" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:9" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="16" t="s">
         <v>58</v>
       </c>
       <c r="C18" s="14"/>
       <c r="D18" s="15"/>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="16" t="s">
         <v>23</v>
       </c>
       <c r="F18" s="15"/>
     </row>
-    <row r="19" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:9" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="16" t="s">
         <v>59</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="15"/>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="16" t="s">
         <v>60</v>
       </c>
       <c r="F19" s="15"/>
     </row>
-    <row r="21" spans="1:9" ht="166" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:9" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="16" t="s">
         <v>62</v>
       </c>
       <c r="C21" s="14"/>
@@ -1141,12 +1171,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="B15:D15"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B14:D14"/>
@@ -1157,6 +1181,12 @@
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="B15:D15"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'TC01'!A1" display="TC01" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -1176,20 +1206,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="56.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1197,7 +1227,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>64</v>
       </c>
@@ -1205,7 +1235,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>65</v>
       </c>
@@ -1213,7 +1243,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>67</v>
       </c>
@@ -1221,7 +1251,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>69</v>
       </c>
@@ -1229,7 +1259,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:3" ht="179.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>71</v>
       </c>
@@ -1237,7 +1267,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>73</v>
       </c>
@@ -1245,7 +1275,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>75</v>
       </c>
@@ -1253,14 +1283,14 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="168" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:3" ht="158.4" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>76</v>
       </c>
@@ -1268,7 +1298,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>77</v>
       </c>
@@ -1276,7 +1306,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>78</v>
       </c>
@@ -1284,7 +1314,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>79</v>
       </c>
@@ -1292,7 +1322,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>80</v>
       </c>
@@ -1300,11 +1330,65 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>81</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="158.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1318,20 +1402,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="56.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1339,7 +1423,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>64</v>
       </c>
@@ -1347,7 +1431,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>65</v>
       </c>
@@ -1355,7 +1439,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>67</v>
       </c>
@@ -1363,7 +1447,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>69</v>
       </c>
@@ -1371,7 +1455,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>71</v>
       </c>
@@ -1379,7 +1463,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>73</v>
       </c>
@@ -1387,7 +1471,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>75</v>
       </c>
@@ -1395,14 +1479,14 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="112" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:3" ht="105.6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>76</v>
       </c>
@@ -1410,7 +1494,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>77</v>
       </c>
@@ -1418,7 +1502,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>78</v>
       </c>
@@ -1426,7 +1510,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>79</v>
       </c>
@@ -1434,7 +1518,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>80</v>
       </c>
@@ -1442,11 +1526,65 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>81</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="105.6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1460,20 +1598,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="56.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1481,7 +1619,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>64</v>
       </c>
@@ -1489,7 +1627,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>65</v>
       </c>
@@ -1497,7 +1635,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>67</v>
       </c>
@@ -1505,7 +1643,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>69</v>
       </c>
@@ -1513,7 +1651,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>71</v>
       </c>
@@ -1521,7 +1659,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>73</v>
       </c>
@@ -1529,7 +1667,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>75</v>
       </c>
@@ -1537,14 +1675,14 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="112" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:3" ht="118.8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>76</v>
       </c>
@@ -1552,7 +1690,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>77</v>
       </c>
@@ -1560,7 +1698,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>78</v>
       </c>
@@ -1568,7 +1706,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>79</v>
       </c>
@@ -1576,7 +1714,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>80</v>
       </c>
@@ -1584,11 +1722,65 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>81</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="118.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="18">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="19" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1602,20 +1794,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="56.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1623,7 +1815,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>64</v>
       </c>
@@ -1631,7 +1823,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>65</v>
       </c>
@@ -1639,7 +1831,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>67</v>
       </c>
@@ -1647,7 +1839,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>69</v>
       </c>
@@ -1655,7 +1847,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>71</v>
       </c>
@@ -1663,7 +1855,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>73</v>
       </c>
@@ -1671,7 +1863,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>75</v>
       </c>
@@ -1679,14 +1871,14 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="56" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:3" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>76</v>
       </c>
@@ -1694,7 +1886,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>77</v>
       </c>
@@ -1702,7 +1894,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>78</v>
       </c>
@@ -1710,7 +1902,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>79</v>
       </c>
@@ -1718,7 +1910,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>80</v>
       </c>
@@ -1726,11 +1918,65 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>81</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="18">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="19" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1744,20 +1990,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="56.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1765,7 +2011,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>64</v>
       </c>
@@ -1773,7 +2019,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>65</v>
       </c>
@@ -1781,7 +2027,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>67</v>
       </c>
@@ -1789,7 +2035,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>69</v>
       </c>
@@ -1797,7 +2043,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>71</v>
       </c>
@@ -1805,7 +2051,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>73</v>
       </c>
@@ -1813,7 +2059,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>75</v>
       </c>
@@ -1821,14 +2067,14 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="84" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:3" ht="79.2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>76</v>
       </c>
@@ -1836,7 +2082,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>77</v>
       </c>
@@ -1844,7 +2090,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>78</v>
       </c>
@@ -1852,7 +2098,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>79</v>
       </c>
@@ -1860,7 +2106,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>80</v>
       </c>
@@ -1868,11 +2114,65 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>81</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="18">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="19" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1886,20 +2186,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="56.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1907,7 +2207,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>64</v>
       </c>
@@ -1915,7 +2215,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>65</v>
       </c>
@@ -1923,7 +2223,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>67</v>
       </c>
@@ -1931,7 +2231,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>69</v>
       </c>
@@ -1939,7 +2239,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>71</v>
       </c>
@@ -1947,7 +2247,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>73</v>
       </c>
@@ -1955,7 +2255,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>75</v>
       </c>
@@ -1963,14 +2263,14 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="84" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:3" ht="79.2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>76</v>
       </c>
@@ -1978,7 +2278,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>77</v>
       </c>
@@ -1986,7 +2286,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>78</v>
       </c>
@@ -1994,7 +2294,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>79</v>
       </c>
@@ -2002,7 +2302,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>80</v>
       </c>
@@ -2010,11 +2310,65 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>81</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="18">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="19" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2028,20 +2382,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="56.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2049,7 +2403,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>64</v>
       </c>
@@ -2057,7 +2411,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>65</v>
       </c>
@@ -2065,7 +2419,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>67</v>
       </c>
@@ -2073,7 +2427,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>69</v>
       </c>
@@ -2081,7 +2435,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>71</v>
       </c>
@@ -2089,7 +2443,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>73</v>
       </c>
@@ -2097,7 +2451,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>75</v>
       </c>
@@ -2105,14 +2459,14 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="70" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:3" ht="66" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>76</v>
       </c>
@@ -2120,7 +2474,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>77</v>
       </c>
@@ -2128,7 +2482,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>78</v>
       </c>
@@ -2136,7 +2490,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>79</v>
       </c>
@@ -2144,7 +2498,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>80</v>
       </c>
@@ -2152,11 +2506,65 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>81</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="66" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="18">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="19" t="s">
         <v>108</v>
       </c>
     </row>

</xml_diff>